<commit_message>
Added density impact experiment
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,27 +429,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>scenario_index</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>
@@ -461,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>28725.35614758425</v>
+        <v>26566.47696253567</v>
       </c>
     </row>
     <row r="3">
@@ -524,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>23963.01774121611</v>
+        <v>10302.47407090168</v>
       </c>
     </row>
     <row r="6">
@@ -587,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>14928.8320178776</v>
+        <v>7519.302316630885</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>29138.17913844815</v>
+        <v>21181.16741521474</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>7284.544784612039</v>
+        <v>5295.291853803686</v>
       </c>
     </row>
     <row r="14">
@@ -713,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>46487.69937914996</v>
+        <v>61076.99869993115</v>
       </c>
     </row>
     <row r="15">
@@ -776,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11621.98641144057</v>
+        <v>13142.63105446239</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
ran density impact experiment
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,27 +417,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>scenario_index</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>
@@ -473,7 +461,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>26566.47696253567</v>
+        <v>19717.4223209293</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +524,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>10302.47407090168</v>
+        <v>14436.5402772733</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +587,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>7519.302316630885</v>
+        <v>6662.640599285361</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +650,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>21181.16741521474</v>
+        <v>23636.05970807384</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +692,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>5295.291853803686</v>
+        <v>5909.014927018459</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +713,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>61076.99869993115</v>
+        <v>30793.55971255575</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +776,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>13142.63105446239</v>
+        <v>19080.47818244137</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Second density impact experiment
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>19717.4223209293</v>
+        <v>22262.85452842836</v>
       </c>
     </row>
     <row r="3">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>14436.5402772733</v>
+        <v>18705.92749495745</v>
       </c>
     </row>
     <row r="6">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>6662.640599285361</v>
+        <v>8581.965522421124</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>23636.05970807384</v>
+        <v>8201.860463743991</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>5909.014927018459</v>
+        <v>2050.465115935998</v>
       </c>
     </row>
     <row r="14">
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>30793.55971255575</v>
+        <v>80843.10694910484</v>
       </c>
     </row>
     <row r="15">
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>19080.47818244137</v>
+        <v>8362.968628543687</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Added explanation to constants, added config path to main files (not experiments, and split model and figures functions
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,27 +429,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>scenario_index</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>
@@ -461,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>22262.85452842836</v>
+        <v>28725.35614758425</v>
       </c>
     </row>
     <row r="3">
@@ -524,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>18705.92749495745</v>
+        <v>23963.01774121611</v>
       </c>
     </row>
     <row r="6">
@@ -587,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>8581.965522421124</v>
+        <v>14928.8320178776</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>8201.860463743991</v>
+        <v>29138.17913844815</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2050.465115935998</v>
+        <v>7284.544784612039</v>
       </c>
     </row>
     <row r="14">
@@ -713,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>80843.10694910484</v>
+        <v>46487.69937914996</v>
       </c>
     </row>
     <row r="15">
@@ -776,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>8362.968628543687</v>
+        <v>11621.98641144057</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
redefined experiment to deterministically solve the problems instead
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios111.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>28725.35614758425</v>
+        <v>38576.00371222453</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>23963.01774121611</v>
+        <v>20009.34735203081</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>14928.8320178776</v>
+        <v>10253.19635316736</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>29138.17913844815</v>
+        <v>13980.483898517</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>7284.544784612039</v>
+        <v>3495.12097462925</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>46487.69937914996</v>
+        <v>61743.18154837705</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11621.98641144057</v>
+        <v>6092.138829340398</v>
       </c>
     </row>
     <row r="18">

</xml_diff>